<commit_message>
feat: tutorial players updated
</commit_message>
<xml_diff>
--- a/configs/Datas/#TutorialBattle.xlsx
+++ b/configs/Datas/#TutorialBattle.xlsx
@@ -133,10 +133,10 @@
     <t>player_sh1ro,player_niko,player_w0nderful,player_makazze</t>
   </si>
   <si>
-    <t>player_zont1x,player_kyousuke,player_im,player_flamez,player_mezii</t>
-  </si>
-  <si>
-    <t>player_magixx,player_teses,player_apex,player_b1t</t>
+    <t>player_zont1x,player_kyousuke,player_im,player_flamez</t>
+  </si>
+  <si>
+    <t>player_magixx,player_teses,player_apex,player_b1t,player_mezii</t>
   </si>
   <si>
     <t>player_chopper,player_kyxsan,player_aleksib</t>

</xml_diff>